<commit_message>
Add filled import template examples
</commit_message>
<xml_diff>
--- a/data/import_template.xlsx
+++ b/data/import_template.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pildymo šablonas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pildymo šablonas'!$A$1:$S$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pildymo šablonas'!$A$1:$S$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -155,8 +155,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImportTemplateTable" displayName="ImportTemplateTable" ref="A1:S2" headerRowCount="1">
-  <autoFilter ref="A1:S2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImportTemplateTable" displayName="ImportTemplateTable" ref="A1:S6" headerRowCount="1">
+  <autoFilter ref="A1:S6"/>
   <tableColumns count="19">
     <tableColumn id="1" name="Įrašo ID"/>
     <tableColumn id="2" name="Įmonės kodas"/>
@@ -471,28 +471,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:S6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="41" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="21" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="17" customWidth="1" min="15" max="15"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="19" customWidth="1" min="13" max="13"/>
+    <col width="19" customWidth="1" min="14" max="14"/>
+    <col width="19" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
-    <col width="29" customWidth="1" min="17" max="17"/>
-    <col width="28" customWidth="1" min="18" max="18"/>
-    <col width="38" customWidth="1" min="19" max="19"/>
+    <col width="41" customWidth="1" min="17" max="17"/>
+    <col width="41" customWidth="1" min="18" max="18"/>
+    <col width="42" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -683,8 +683,376 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>pvz-betono-centras-vilnius</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>123018186</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>UAB Betono centras</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Betono centras</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Vilnius</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Vilniaus m. sav.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Naujoji Riovonių g. 11, Vilnius</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>54.6560815</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>25.2314767</v>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Stetter</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>2x3,35 m³</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>100 m³/val.</t>
+        </is>
+      </c>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>Viešai skelbiamas Betono centro betono mazgas Vilniuje.</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>https://betonocentras.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>https://betonocentras.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>Pavyzdinė eilutė iš esamų duomenų; trūkstami techniniai duomenys pažymėti aiškiai.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>pvz-betono-centras-klaipeda</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>123018186</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>UAB Betono centras</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Betono centras</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Klaipėda</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Klaipėdos m. sav.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Liepų g. 87N, Klaipėda</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>55.7290357</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>21.1544709</v>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Klaipėdos betono mazgas</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>Viešai skelbiamas Betono centro betono mazgas Klaipėdoje.</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>https://betonocentras.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>https://betonocentras.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>Pavyzdinė eilutė iš esamų duomenų; parodyta, kaip pildyti eilutę, kai dalis techninių duomenų nerasta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>pvz-transdosa-druskininkai</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>UAB Transdosa</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Transdosa</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Druskininkai</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Druskininkų sav.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Žvyro g. 2A, Margų k., Druskininkų sav.</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>54.146785</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>23.9291769</v>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Elkomix-90 quick master</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>1,5 m³</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>40 m³/h</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>Viešai skelbiamas betono mišinių tiekėjas Druskininkų regione.</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.transdosa.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.transdosa.lt/betonas/</t>
+        </is>
+      </c>
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>Techniniai mazgo duomenys įrašyti pagal naudotojo pateiktą informaciją.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>pvz-telsiu-keliai-telsiai</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>180200843</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>UAB Telšių keliai</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Telšių keliai</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Telšiai</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Telšių r. sav.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Mažeikių g. 18, Telšiai</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>56.0004158</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>22.2581129</v>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Elkon</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>Oficialiame įmonės puslapyje skelbiama betono mišinių gamyba ir prekyba.</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr">
+        <is>
+          <t>Įtraukta pagal naudotojo informaciją; veikla patvirtinta oficialiame lietuviškame įmonės puslapyje.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S2"/>
+  <autoFilter ref="A1:S6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>